<commit_message>
chore: update test data files and generators to include Cluster column across all test folders
</commit_message>
<xml_diff>
--- a/backend/excel-templates/New-Test-data/bachelor_bct_test_data.xlsx
+++ b/backend/excel-templates/New-Test-data/bachelor_bct_test_data.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -416,9 +416,12 @@
         <v>Batch</v>
       </c>
       <c r="F1" t="str">
+        <v>Cluster</v>
+      </c>
+      <c r="G1" t="str">
         <v>Supervisor</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>External Examiner</v>
       </c>
     </row>
@@ -439,9 +442,12 @@
         <v>083</v>
       </c>
       <c r="F2" t="str">
+        <v>AIML</v>
+      </c>
+      <c r="G2" t="str">
         <v>Prof. Dr. Dinesh Koirala</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>Dr. Anisha Rana</v>
       </c>
     </row>
@@ -462,9 +468,12 @@
         <v>083</v>
       </c>
       <c r="F3" t="str">
+        <v>IPCV</v>
+      </c>
+      <c r="G3" t="str">
         <v>Assoc. Prof. Dr. Meena Shrestha</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>Dr. Bidur Khadka</v>
       </c>
     </row>
@@ -485,9 +494,12 @@
         <v>083</v>
       </c>
       <c r="F4" t="str">
+        <v>ANLP</v>
+      </c>
+      <c r="G4" t="str">
         <v>Dr. Kiran Adhikari</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>Assoc. Prof. Dr. Manisha Aryal</v>
       </c>
     </row>
@@ -508,9 +520,12 @@
         <v>083</v>
       </c>
       <c r="F5" t="str">
+        <v>NTS</v>
+      </c>
+      <c r="G5" t="str">
         <v/>
       </c>
-      <c r="G5" t="str">
+      <c r="H5" t="str">
         <v>Dr. Sabin Wagle</v>
       </c>
     </row>
@@ -531,15 +546,18 @@
         <v>083</v>
       </c>
       <c r="F6" t="str">
+        <v>EDMES</v>
+      </c>
+      <c r="G6" t="str">
         <v>Dr. Nilima Joshi</v>
       </c>
-      <c r="G6" t="str">
+      <c r="H6" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>